<commit_message>
Updated MJ email thing
</commit_message>
<xml_diff>
--- a/Processed PO Numbers.xlsx
+++ b/Processed PO Numbers.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <x:fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <x:fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <x:workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DigitalDoorLocks-Aut\Documents\UiPath\(Task 37) Harvey Norman Order processing Automation\Harvey Norman Order Processing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFA930D7-A9EC-405F-9476-49E0DFC1D8C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{612550DB-9B71-43E7-84F7-ED8840FE4B76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <x:bookViews>
     <x:workbookView xWindow="-120" yWindow="-120" windowWidth="30960" windowHeight="16800" firstSheet="0" activeTab="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </x:bookViews>
@@ -16,7 +16,7 @@
     <x:sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </x:sheets>
   <x:definedNames>
-    <x:definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$A$12</x:definedName>
+    <x:definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$A$11</x:definedName>
   </x:definedNames>
   <x:calcPr calcId="162913"/>
   <x:extLst>
@@ -39,238 +39,370 @@
     <x:t>Status</x:t>
   </x:si>
   <x:si>
-    <x:t>70127(0123560)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00021957</x:t>
+    <x:t>357858(0106160)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00021958</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Completed</x:t>
+  </x:si>
+  <x:si>
+    <x:t>214677(0120660)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00021959</x:t>
+  </x:si>
+  <x:si>
+    <x:t>350084(0116760)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00021960</x:t>
+  </x:si>
+  <x:si>
+    <x:t>30011(0113360)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022020</x:t>
+  </x:si>
+  <x:si>
+    <x:t>245986(0105460)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022021</x:t>
+  </x:si>
+  <x:si>
+    <x:t>214889(0120660)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022022</x:t>
+  </x:si>
+  <x:si>
+    <x:t>158949(0116860)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022023</x:t>
+  </x:si>
+  <x:si>
+    <x:t>101610(0120860)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022025</x:t>
+  </x:si>
+  <x:si>
+    <x:t>167542(0121660)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>191981(5003860)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022027</x:t>
+  </x:si>
+  <x:si>
+    <x:t>943397(133725)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022047</x:t>
+  </x:si>
+  <x:si>
+    <x:t>218328(0114360)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022080</x:t>
+  </x:si>
+  <x:si>
+    <x:t>350683(0116760)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022081</x:t>
+  </x:si>
+  <x:si>
+    <x:t>14917(0127860)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022082</x:t>
+  </x:si>
+  <x:si>
+    <x:t>343338(0105660)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022091</x:t>
+  </x:si>
+  <x:si>
+    <x:t>215102(0120660)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022092</x:t>
+  </x:si>
+  <x:si>
+    <x:t>368154(0102160)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022128</x:t>
+  </x:si>
+  <x:si>
+    <x:t>499150(0102060)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022129</x:t>
+  </x:si>
+  <x:si>
+    <x:t>247034(0113860)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022130</x:t>
+  </x:si>
+  <x:si>
+    <x:t>309992(0112860)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022131</x:t>
+  </x:si>
+  <x:si>
+    <x:t>266051(0109760)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022132</x:t>
+  </x:si>
+  <x:si>
+    <x:t>196927(0163760)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022134</x:t>
+  </x:si>
+  <x:si>
+    <x:t>293319(0108860)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022135</x:t>
+  </x:si>
+  <x:si>
+    <x:t>101865(0120860)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022146</x:t>
+  </x:si>
+  <x:si>
+    <x:t>77218(0119760)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022147</x:t>
+  </x:si>
+  <x:si>
+    <x:t>421818(109260)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022151</x:t>
+  </x:si>
+  <x:si>
+    <x:t>60317(0125160)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022152</x:t>
+  </x:si>
+  <x:si>
+    <x:t>308312(0104460)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022153</x:t>
+  </x:si>
+  <x:si>
+    <x:t>358566(0106160)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022154</x:t>
+  </x:si>
+  <x:si>
+    <x:t>499485(0102060)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022195</x:t>
+  </x:si>
+  <x:si>
+    <x:t>281788(0104060)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022196</x:t>
+  </x:si>
+  <x:si>
+    <x:t>449581(0102860)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022197</x:t>
+  </x:si>
+  <x:si>
+    <x:t>215931(0115960)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022206</x:t>
+  </x:si>
+  <x:si>
+    <x:t>434129(0107560)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022207</x:t>
+  </x:si>
+  <x:si>
+    <x:t>215536(0120660)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022224</x:t>
+  </x:si>
+  <x:si>
+    <x:t>359019(0106160)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022266</x:t>
+  </x:si>
+  <x:si>
+    <x:t>102405(0120860)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022365</x:t>
+  </x:si>
+  <x:si>
+    <x:t>209611(0103860)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022366</x:t>
+  </x:si>
+  <x:si>
+    <x:t>434844(0107560)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022368</x:t>
+  </x:si>
+  <x:si>
+    <x:t>450525(0102860)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022373</x:t>
+  </x:si>
+  <x:si>
+    <x:t>409351(0109660)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022411</x:t>
+  </x:si>
+  <x:si>
+    <x:t>344920(0105660)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022412</x:t>
+  </x:si>
+  <x:si>
+    <x:t>198036(0163760)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022413</x:t>
+  </x:si>
+  <x:si>
+    <x:t>352641(0116760)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022439</x:t>
+  </x:si>
+  <x:si>
+    <x:t>352937(0116760)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022467</x:t>
+  </x:si>
+  <x:si>
+    <x:t>247684(0113860)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022468</x:t>
+  </x:si>
+  <x:si>
+    <x:t>216625(0120660)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022469</x:t>
+  </x:si>
+  <x:si>
+    <x:t>338651(0107960)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022500</x:t>
+  </x:si>
+  <x:si>
+    <x:t>160109(0116860)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022514</x:t>
+  </x:si>
+  <x:si>
+    <x:t>4105135520(0128960)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022521</x:t>
+  </x:si>
+  <x:si>
+    <x:t>204282(0117860)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022540</x:t>
+  </x:si>
+  <x:si>
+    <x:t>16325(0127860)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022541</x:t>
+  </x:si>
+  <x:si>
+    <x:t>297644(0162662)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022542</x:t>
+  </x:si>
+  <x:si>
+    <x:t>13490(0146160)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022543</x:t>
+  </x:si>
+  <x:si>
+    <x:t>424186(109260)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022567</x:t>
+  </x:si>
+  <x:si>
+    <x:t>216896(0120660)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022584</x:t>
+  </x:si>
+  <x:si>
+    <x:t>245718(0120360)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022585</x:t>
+  </x:si>
+  <x:si>
+    <x:t>198615(0102560)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022586</x:t>
+  </x:si>
+  <x:si>
+    <x:t>162420(0118860)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00022622</x:t>
+  </x:si>
+  <x:si>
+    <x:t>362720(0106160)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SO-00023087</x:t>
   </x:si>
   <x:si>
     <x:t>Skipped</x:t>
-  </x:si>
-  <x:si>
-    <x:t>357858(0106160)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00021958</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Completed</x:t>
-  </x:si>
-  <x:si>
-    <x:t>214677(0120660)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00021959</x:t>
-  </x:si>
-  <x:si>
-    <x:t>350084(0116760)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00021960</x:t>
-  </x:si>
-  <x:si>
-    <x:t>30011(0113360)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022020</x:t>
-  </x:si>
-  <x:si>
-    <x:t>245986(0105460)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022021</x:t>
-  </x:si>
-  <x:si>
-    <x:t>214889(0120660)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022022</x:t>
-  </x:si>
-  <x:si>
-    <x:t>158949(0116860)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022023</x:t>
-  </x:si>
-  <x:si>
-    <x:t>101610(0120860)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022025</x:t>
-  </x:si>
-  <x:si>
-    <x:t>167542(0121660)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>191981(5003860)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022027</x:t>
-  </x:si>
-  <x:si>
-    <x:t>943397(133725)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022047</x:t>
-  </x:si>
-  <x:si>
-    <x:t>421677(0109160)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022067</x:t>
-  </x:si>
-  <x:si>
-    <x:t>218328(0114360)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022080</x:t>
-  </x:si>
-  <x:si>
-    <x:t>350683(0116760)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022081</x:t>
-  </x:si>
-  <x:si>
-    <x:t>14917(0127860)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022082</x:t>
-  </x:si>
-  <x:si>
-    <x:t>343338(0105660)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022091</x:t>
-  </x:si>
-  <x:si>
-    <x:t>215102(0120660)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022092</x:t>
-  </x:si>
-  <x:si>
-    <x:t>368154(0102160)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022128</x:t>
-  </x:si>
-  <x:si>
-    <x:t>499150(0102060)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022129</x:t>
-  </x:si>
-  <x:si>
-    <x:t>247034(0113860)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022130</x:t>
-  </x:si>
-  <x:si>
-    <x:t>309992(0112860)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022131</x:t>
-  </x:si>
-  <x:si>
-    <x:t>266051(0109760)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022132</x:t>
-  </x:si>
-  <x:si>
-    <x:t>196927(0163760)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022134</x:t>
-  </x:si>
-  <x:si>
-    <x:t>293319(0108860)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022135</x:t>
-  </x:si>
-  <x:si>
-    <x:t>101865(0120860)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022146</x:t>
-  </x:si>
-  <x:si>
-    <x:t>77218(0119760)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022147</x:t>
-  </x:si>
-  <x:si>
-    <x:t>421818(109260)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022151</x:t>
-  </x:si>
-  <x:si>
-    <x:t>60317(0125160)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022152</x:t>
-  </x:si>
-  <x:si>
-    <x:t>308312(0104460)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022153</x:t>
-  </x:si>
-  <x:si>
-    <x:t>358566(0106160)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022154</x:t>
-  </x:si>
-  <x:si>
-    <x:t>499485(0102060)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022195</x:t>
-  </x:si>
-  <x:si>
-    <x:t>281788(0104060)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022196</x:t>
-  </x:si>
-  <x:si>
-    <x:t>449581(0102860)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022197</x:t>
-  </x:si>
-  <x:si>
-    <x:t>215931(0115960)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022206</x:t>
-  </x:si>
-  <x:si>
-    <x:t>434129(0107560)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022207</x:t>
-  </x:si>
-  <x:si>
-    <x:t>215536(0120660)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022224</x:t>
-  </x:si>
-  <x:si>
-    <x:t>359019(0106160)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SO-00022266</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -600,7 +732,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C38"/>
+  <x:dimension ref="A1:C60"/>
   <x:sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <x:cols>
     <x:col min="1" max="1" width="16.425781" style="0" bestFit="1" customWidth="1"/>
@@ -638,125 +770,125 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A4" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="B4" s="0" t="s">
-        <x:v>10</x:v>
-      </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A5" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="B5" s="0" t="s">
-        <x:v>12</x:v>
-      </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A6" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B6" s="0" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="B6" s="0" t="s">
-        <x:v>14</x:v>
-      </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A7" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B7" s="0" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="B7" s="0" t="s">
-        <x:v>16</x:v>
-      </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A8" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B8" s="0" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="B8" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
       <x:c r="C8" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A9" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B9" s="0" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="B9" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
       <x:c r="C9" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A10" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B10" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="B10" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="C10" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A11" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B11" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="B11" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
       <x:c r="C11" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A12" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="B12" s="0" t="s">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="B12" s="0" t="s">
-        <x:v>26</x:v>
-      </x:c>
       <x:c r="C12" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A13" s="0" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B13" s="0" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="B13" s="0" t="s">
-        <x:v>28</x:v>
-      </x:c>
       <x:c r="C13" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A14" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B14" s="0" t="s">
         <x:v>29</x:v>
-      </x:c>
-      <x:c r="B14" s="0" t="s">
-        <x:v>30</x:v>
       </x:c>
       <x:c r="C14" s="0" t="s">
         <x:v>5</x:v>
@@ -764,281 +896,523 @@
     </x:row>
     <x:row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A15" s="0" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B15" s="0" t="s">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="B15" s="0" t="s">
-        <x:v>32</x:v>
-      </x:c>
       <x:c r="C15" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A16" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B16" s="0" t="s">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="B16" s="0" t="s">
-        <x:v>34</x:v>
-      </x:c>
       <x:c r="C16" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A17" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B17" s="0" t="s">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="B17" s="0" t="s">
-        <x:v>36</x:v>
-      </x:c>
       <x:c r="C17" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A18" s="0" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="B18" s="0" t="s">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="B18" s="0" t="s">
-        <x:v>38</x:v>
-      </x:c>
       <x:c r="C18" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A19" s="0" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="B19" s="0" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="B19" s="0" t="s">
-        <x:v>40</x:v>
-      </x:c>
       <x:c r="C19" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A20" s="0" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="B20" s="0" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="B20" s="0" t="s">
-        <x:v>42</x:v>
-      </x:c>
       <x:c r="C20" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A21" s="0" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="B21" s="0" t="s">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="B21" s="0" t="s">
-        <x:v>44</x:v>
-      </x:c>
       <x:c r="C21" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A22" s="0" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="B22" s="0" t="s">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="B22" s="0" t="s">
-        <x:v>46</x:v>
-      </x:c>
       <x:c r="C22" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A23" s="0" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="B23" s="0" t="s">
         <x:v>47</x:v>
       </x:c>
-      <x:c r="B23" s="0" t="s">
-        <x:v>48</x:v>
-      </x:c>
       <x:c r="C23" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A24" s="0" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="B24" s="0" t="s">
         <x:v>49</x:v>
       </x:c>
-      <x:c r="B24" s="0" t="s">
-        <x:v>50</x:v>
-      </x:c>
       <x:c r="C24" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A25" s="0" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="B25" s="0" t="s">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="B25" s="0" t="s">
-        <x:v>52</x:v>
-      </x:c>
       <x:c r="C25" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A26" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="B26" s="0" t="s">
         <x:v>53</x:v>
       </x:c>
-      <x:c r="B26" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
       <x:c r="C26" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A27" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="B27" s="0" t="s">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="B27" s="0" t="s">
-        <x:v>56</x:v>
-      </x:c>
       <x:c r="C27" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A28" s="0" t="s">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="B28" s="0" t="s">
         <x:v>57</x:v>
       </x:c>
-      <x:c r="B28" s="0" t="s">
-        <x:v>58</x:v>
-      </x:c>
       <x:c r="C28" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A29" s="0" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="B29" s="0" t="s">
         <x:v>59</x:v>
       </x:c>
-      <x:c r="B29" s="0" t="s">
-        <x:v>60</x:v>
-      </x:c>
       <x:c r="C29" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A30" s="0" t="s">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="B30" s="0" t="s">
         <x:v>61</x:v>
       </x:c>
-      <x:c r="B30" s="0" t="s">
-        <x:v>62</x:v>
-      </x:c>
       <x:c r="C30" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A31" s="0" t="s">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="B31" s="0" t="s">
         <x:v>63</x:v>
       </x:c>
-      <x:c r="B31" s="0" t="s">
-        <x:v>64</x:v>
-      </x:c>
       <x:c r="C31" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A32" s="0" t="s">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B32" s="0" t="s">
         <x:v>65</x:v>
       </x:c>
-      <x:c r="B32" s="0" t="s">
-        <x:v>66</x:v>
-      </x:c>
       <x:c r="C32" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A33" s="0" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="B33" s="0" t="s">
         <x:v>67</x:v>
       </x:c>
-      <x:c r="B33" s="0" t="s">
-        <x:v>68</x:v>
-      </x:c>
       <x:c r="C33" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A34" s="0" t="s">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="B34" s="0" t="s">
         <x:v>69</x:v>
       </x:c>
-      <x:c r="B34" s="0" t="s">
-        <x:v>70</x:v>
-      </x:c>
       <x:c r="C34" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A35" s="0" t="s">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="B35" s="0" t="s">
         <x:v>71</x:v>
       </x:c>
-      <x:c r="B35" s="0" t="s">
-        <x:v>72</x:v>
-      </x:c>
       <x:c r="C35" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A36" s="0" t="s">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="B36" s="0" t="s">
         <x:v>73</x:v>
       </x:c>
-      <x:c r="B36" s="0" t="s">
-        <x:v>74</x:v>
-      </x:c>
       <x:c r="C36" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A37" s="0" t="s">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="B37" s="0" t="s">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="B37" s="0" t="s">
-        <x:v>76</x:v>
-      </x:c>
       <x:c r="C37" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <x:c r="A38" s="0" t="s">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="B38" s="0" t="s">
         <x:v>77</x:v>
       </x:c>
-      <x:c r="B38" s="0" t="s">
+      <x:c r="C38" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <x:c r="A39" s="0" t="s">
         <x:v>78</x:v>
       </x:c>
-      <x:c r="C38" s="0" t="s">
-        <x:v>8</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39" spans="1:3">
-      <x:c r="A39" s="0" t="s">
+      <x:c r="B39" s="0" t="s">
         <x:v>79</x:v>
       </x:c>
-      <x:c r="B39" s="0" t="s">
+      <x:c r="C39" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <x:c r="A40" s="0" t="s">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="C39" s="0" t="s">
-        <x:v>5</x:v>
+      <x:c r="B40" s="0" t="s">
+        <x:v>81</x:v>
+      </x:c>
+      <x:c r="C40" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <x:c r="A41" s="0" t="s">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="B41" s="0" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="C41" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <x:c r="A42" s="0" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="B42" s="0" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="C42" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <x:c r="A43" s="0" t="s">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="B43" s="0" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="C43" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <x:c r="A44" s="0" t="s">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="B44" s="0" t="s">
+        <x:v>89</x:v>
+      </x:c>
+      <x:c r="C44" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <x:c r="A45" s="0" t="s">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="B45" s="0" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="C45" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <x:c r="A46" s="0" t="s">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="B46" s="0" t="s">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="C46" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <x:c r="A47" s="0" t="s">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="B47" s="0" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="C47" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <x:c r="A48" s="0" t="s">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="B48" s="0" t="s">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="C48" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <x:c r="A49" s="0" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="B49" s="0" t="s">
+        <x:v>99</x:v>
+      </x:c>
+      <x:c r="C49" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <x:c r="A50" s="0" t="s">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="B50" s="0" t="s">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="C50" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <x:c r="A51" s="0" t="s">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="B51" s="0" t="s">
+        <x:v>103</x:v>
+      </x:c>
+      <x:c r="C51" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <x:c r="A52" s="0" t="s">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="B52" s="0" t="s">
+        <x:v>105</x:v>
+      </x:c>
+      <x:c r="C52" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <x:c r="A53" s="0" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="B53" s="0" t="s">
+        <x:v>107</x:v>
+      </x:c>
+      <x:c r="C53" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <x:c r="A54" s="0" t="s">
+        <x:v>108</x:v>
+      </x:c>
+      <x:c r="B54" s="0" t="s">
+        <x:v>109</x:v>
+      </x:c>
+      <x:c r="C54" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <x:c r="A55" s="0" t="s">
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="B55" s="0" t="s">
+        <x:v>111</x:v>
+      </x:c>
+      <x:c r="C55" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <x:c r="A56" s="0" t="s">
+        <x:v>112</x:v>
+      </x:c>
+      <x:c r="B56" s="0" t="s">
+        <x:v>113</x:v>
+      </x:c>
+      <x:c r="C56" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <x:c r="A57" s="0" t="s">
+        <x:v>114</x:v>
+      </x:c>
+      <x:c r="B57" s="0" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="C57" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <x:c r="A58" s="0" t="s">
+        <x:v>116</x:v>
+      </x:c>
+      <x:c r="B58" s="0" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="C58" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <x:c r="A59" s="0" t="s">
+        <x:v>118</x:v>
+      </x:c>
+      <x:c r="B59" s="0" t="s">
+        <x:v>119</x:v>
+      </x:c>
+      <x:c r="C59" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <x:c r="A60" s="0" t="s">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="B60" s="0" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="C60" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" spans="1:3">
+      <x:c r="A61" s="0" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="B61" s="0" t="s">
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="C61" s="0" t="s">
+        <x:v>124</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:autoFilter ref="A1:A12"/>
+  <x:autoFilter ref="A1:A11"/>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="portrait" blackAndWhite="0" draft="0" cellComments="none" errors="displayed" r:id="rId1"/>

</xml_diff>